<commit_message>
Rimuovi Oshina dal foglio costi personale domestico
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JqwGFxpn8nXJFHoUJvfu6N
</commit_message>
<xml_diff>
--- a/personale-domestico/costi-personale-domestico.xlsx
+++ b/personale-domestico/costi-personale-domestico.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="107">
   <si>
     <t xml:space="preserve">Personale di casa – costo reale (pagamento in contanti, senza contratto)</t>
   </si>
@@ -53,12 +53,6 @@
   </si>
   <si>
     <t xml:space="preserve">% sul totale</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oshina</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Colf</t>
   </si>
   <si>
     <t xml:space="preserve">Elisa</t>
@@ -901,7 +895,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42"/>
@@ -956,26 +950,26 @@
         <v>11</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>11.5</v>
+        <v>12</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E5" s="7" t="n">
         <f aca="false">C5*D5</f>
-        <v>103.5</v>
+        <v>72</v>
       </c>
       <c r="F5" s="7" t="n">
         <f aca="false">E5*Parametri!$B$6/Parametri!$B$7</f>
-        <v>448.5</v>
+        <v>312</v>
       </c>
       <c r="G5" s="8" t="n">
         <f aca="false">E5*Parametri!$B$6</f>
-        <v>5382</v>
+        <v>3744</v>
       </c>
       <c r="H5" s="9" t="n">
-        <f aca="false">IF($G$8=0,0,G5/$G$8)</f>
-        <v>0.480278422273782</v>
+        <f aca="false">IF($G$7=0,0,G5/$G$7)</f>
+        <v>0.642857142857143</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -983,159 +977,129 @@
         <v>12</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E6" s="7" t="n">
         <f aca="false">C6*D6</f>
-        <v>72</v>
+        <v>40</v>
       </c>
       <c r="F6" s="7" t="n">
         <f aca="false">E6*Parametri!$B$6/Parametri!$B$7</f>
-        <v>312</v>
+        <v>173.333333333333</v>
       </c>
       <c r="G6" s="8" t="n">
         <f aca="false">E6*Parametri!$B$6</f>
-        <v>3744</v>
+        <v>2080</v>
       </c>
       <c r="H6" s="9" t="n">
-        <f aca="false">IF($G$8=0,0,G6/$G$8)</f>
-        <v>0.334106728538283</v>
+        <f aca="false">IF($G$7=0,0,G6/$G$7)</f>
+        <v>0.357142857142857</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="10"/>
+      <c r="C7" s="11" t="n">
+        <f aca="false">IF(D7=0,0,E7/D7)</f>
+        <v>11.2</v>
+      </c>
+      <c r="D7" s="12" t="n">
+        <f aca="false">SUM(D5:D6)</f>
+        <v>10</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <f aca="false">SUM(E5:E6)</f>
+        <v>112</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <f aca="false">SUM(F5:F6)</f>
+        <v>485.333333333333</v>
+      </c>
+      <c r="G7" s="11" t="n">
+        <f aca="false">SUM(G5:G6)</f>
+        <v>5824</v>
+      </c>
+      <c r="H7" s="13" t="n">
+        <f aca="false">SUM(H5:H6)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="D7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="E7" s="7" t="n">
-        <f aca="false">C7*D7</f>
-        <v>40</v>
-      </c>
-      <c r="F7" s="7" t="n">
-        <f aca="false">E7*Parametri!$B$6/Parametri!$B$7</f>
-        <v>173.333333333333</v>
-      </c>
-      <c r="G7" s="8" t="n">
-        <f aca="false">E7*Parametri!$B$6</f>
-        <v>2080</v>
-      </c>
-      <c r="H7" s="9" t="n">
-        <f aca="false">IF($G$8=0,0,G7/$G$8)</f>
-        <v>0.185614849187935</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="s">
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="10"/>
-      <c r="C8" s="11" t="n">
-        <f aca="false">IF(D8=0,0,E8/D8)</f>
-        <v>11.3421052631579</v>
-      </c>
-      <c r="D8" s="12" t="n">
-        <f aca="false">SUM(D5:D7)</f>
-        <v>19</v>
-      </c>
-      <c r="E8" s="11" t="n">
-        <f aca="false">SUM(E5:E7)</f>
-        <v>215.5</v>
-      </c>
-      <c r="F8" s="11" t="n">
-        <f aca="false">SUM(F5:F7)</f>
-        <v>933.833333333333</v>
-      </c>
-      <c r="G8" s="11" t="n">
-        <f aca="false">SUM(G5:G7)</f>
-        <v>11206</v>
-      </c>
-      <c r="H8" s="13" t="n">
-        <f aca="false">SUM(H5:H7)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="14" t="s">
-        <v>16</v>
+      <c r="B11" s="8" t="n">
+        <f aca="false">F7</f>
+        <v>485.333333333333</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B12" s="8" t="n">
-        <f aca="false">F8</f>
-        <v>933.833333333333</v>
+        <f aca="false">E7*5</f>
+        <v>560</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="15" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B13" s="8" t="n">
-        <f aca="false">E8*5</f>
-        <v>1077.5</v>
+        <f aca="false">E7*4</f>
+        <v>448</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="B14" s="8" t="n">
-        <f aca="false">E8*4</f>
-        <v>862</v>
+        <v>18</v>
+      </c>
+      <c r="B14" s="16" t="n">
+        <f aca="false">D7*Parametri!$B$6</f>
+        <v>520</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="B15" s="8" t="n">
+        <f aca="false">C7</f>
+        <v>11.2</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="B15" s="16" t="n">
-        <f aca="false">D8*Parametri!$B$6</f>
-        <v>988</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="15" t="s">
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="17" t="s">
         <v>21</v>
-      </c>
-      <c r="B16" s="8" t="n">
-        <f aca="false">C8</f>
-        <v>11.3421052631579</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="14" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="17" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="17" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="17" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -1165,50 +1129,50 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>28</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B5" s="18" t="n">
         <v>2027</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B6" s="18" t="n">
         <v>52</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B7" s="18" t="n">
         <v>12</v>
@@ -1217,86 +1181,86 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="15" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B12" s="18" t="n">
         <v>52</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="15" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B13" s="18" t="n">
         <v>1</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="15" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B14" s="6" t="n">
         <v>13.5</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="15" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B15" s="20" t="n">
         <v>0.06</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C20" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="D20" s="3" t="s">
         <v>49</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1310,7 +1274,7 @@
         <v>0.43</v>
       </c>
       <c r="D21" s="15" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1324,7 +1288,7 @@
         <v>0.48</v>
       </c>
       <c r="D22" s="15" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1338,12 +1302,12 @@
         <v>0.59</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="15" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B24" s="20" t="n">
         <v>1.24</v>
@@ -1352,12 +1316,12 @@
         <v>0.31</v>
       </c>
       <c r="D24" s="15" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -1376,7 +1340,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J58"/>
+  <dimension ref="A1:J46"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -1392,20 +1356,20 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>2</v>
@@ -1414,47 +1378,47 @@
         <v>4</v>
       </c>
       <c r="E4" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="G4" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="H4" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="I4" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="H4" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>66</v>
-      </c>
       <c r="J4" s="3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B5" s="21" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="22" t="str">
         <f aca="false">Riepilogo!$A$5</f>
-        <v>Oshina</v>
+        <v>Elisa</v>
       </c>
       <c r="D5" s="23" t="n">
         <f aca="false">Riepilogo!$C$5</f>
-        <v>11.5</v>
+        <v>12</v>
       </c>
       <c r="E5" s="24" t="n">
         <f aca="false">Riepilogo!$D$5*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B5,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B5+1,0))))</f>
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="F5" s="6"/>
       <c r="G5" s="7" t="n">
         <f aca="false">IF(F5="",E5,F5)*D5</f>
-        <v>414</v>
+        <v>288</v>
       </c>
       <c r="H5" s="25"/>
       <c r="I5" s="4"/>
@@ -1462,27 +1426,27 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B6" s="21" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="22" t="str">
         <f aca="false">Riepilogo!$A$6</f>
-        <v>Elisa</v>
+        <v>Corina</v>
       </c>
       <c r="D6" s="23" t="n">
         <f aca="false">Riepilogo!$C$6</f>
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E6" s="24" t="n">
         <f aca="false">Riepilogo!$D$6*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B6,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B6+1,0))))</f>
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="F6" s="6"/>
       <c r="G6" s="7" t="n">
         <f aca="false">IF(F6="",E6,F6)*D6</f>
-        <v>288</v>
+        <v>160</v>
       </c>
       <c r="H6" s="25"/>
       <c r="I6" s="4"/>
@@ -1490,27 +1454,27 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B7" s="21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C7" s="22" t="str">
-        <f aca="false">Riepilogo!$A$7</f>
-        <v>Corina</v>
+        <f aca="false">Riepilogo!$A$5</f>
+        <v>Elisa</v>
       </c>
       <c r="D7" s="23" t="n">
-        <f aca="false">Riepilogo!$C$7</f>
-        <v>10</v>
+        <f aca="false">Riepilogo!$C$5</f>
+        <v>12</v>
       </c>
       <c r="E7" s="24" t="n">
-        <f aca="false">Riepilogo!$D$7*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B7,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B7+1,0))))</f>
-        <v>16</v>
+        <f aca="false">Riepilogo!$D$5*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B7,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B7+1,0))))</f>
+        <v>24</v>
       </c>
       <c r="F7" s="6"/>
       <c r="G7" s="7" t="n">
         <f aca="false">IF(F7="",E7,F7)*D7</f>
-        <v>160</v>
+        <v>288</v>
       </c>
       <c r="H7" s="25"/>
       <c r="I7" s="4"/>
@@ -1518,27 +1482,27 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B8" s="21" t="n">
         <v>2</v>
       </c>
       <c r="C8" s="22" t="str">
-        <f aca="false">Riepilogo!$A$5</f>
-        <v>Oshina</v>
+        <f aca="false">Riepilogo!$A$6</f>
+        <v>Corina</v>
       </c>
       <c r="D8" s="23" t="n">
-        <f aca="false">Riepilogo!$C$5</f>
-        <v>11.5</v>
+        <f aca="false">Riepilogo!$C$6</f>
+        <v>10</v>
       </c>
       <c r="E8" s="24" t="n">
-        <f aca="false">Riepilogo!$D$5*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B8,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B8+1,0))))</f>
-        <v>36</v>
+        <f aca="false">Riepilogo!$D$6*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B8,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B8+1,0))))</f>
+        <v>16</v>
       </c>
       <c r="F8" s="6"/>
       <c r="G8" s="7" t="n">
         <f aca="false">IF(F8="",E8,F8)*D8</f>
-        <v>414</v>
+        <v>160</v>
       </c>
       <c r="H8" s="25"/>
       <c r="I8" s="4"/>
@@ -1546,27 +1510,27 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B9" s="21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C9" s="22" t="str">
-        <f aca="false">Riepilogo!$A$6</f>
+        <f aca="false">Riepilogo!$A$5</f>
         <v>Elisa</v>
       </c>
       <c r="D9" s="23" t="n">
-        <f aca="false">Riepilogo!$C$6</f>
+        <f aca="false">Riepilogo!$C$5</f>
         <v>12</v>
       </c>
       <c r="E9" s="24" t="n">
-        <f aca="false">Riepilogo!$D$6*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B9,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B9+1,0))))</f>
-        <v>24</v>
+        <f aca="false">Riepilogo!$D$5*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B9,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B9+1,0))))</f>
+        <v>30</v>
       </c>
       <c r="F9" s="6"/>
       <c r="G9" s="7" t="n">
         <f aca="false">IF(F9="",E9,F9)*D9</f>
-        <v>288</v>
+        <v>360</v>
       </c>
       <c r="H9" s="25"/>
       <c r="I9" s="4"/>
@@ -1574,27 +1538,27 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B10" s="21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C10" s="22" t="str">
-        <f aca="false">Riepilogo!$A$7</f>
+        <f aca="false">Riepilogo!$A$6</f>
         <v>Corina</v>
       </c>
       <c r="D10" s="23" t="n">
-        <f aca="false">Riepilogo!$C$7</f>
+        <f aca="false">Riepilogo!$C$6</f>
         <v>10</v>
       </c>
       <c r="E10" s="24" t="n">
-        <f aca="false">Riepilogo!$D$7*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B10,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B10+1,0))))</f>
-        <v>16</v>
+        <f aca="false">Riepilogo!$D$6*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B10,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B10+1,0))))</f>
+        <v>20</v>
       </c>
       <c r="F10" s="6"/>
       <c r="G10" s="7" t="n">
         <f aca="false">IF(F10="",E10,F10)*D10</f>
-        <v>160</v>
+        <v>200</v>
       </c>
       <c r="H10" s="25"/>
       <c r="I10" s="4"/>
@@ -1602,27 +1566,27 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B11" s="21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C11" s="22" t="str">
         <f aca="false">Riepilogo!$A$5</f>
-        <v>Oshina</v>
+        <v>Elisa</v>
       </c>
       <c r="D11" s="23" t="n">
         <f aca="false">Riepilogo!$C$5</f>
-        <v>11.5</v>
+        <v>12</v>
       </c>
       <c r="E11" s="24" t="n">
         <f aca="false">Riepilogo!$D$5*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B11,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B11+1,0))))</f>
-        <v>45</v>
+        <v>24</v>
       </c>
       <c r="F11" s="6"/>
       <c r="G11" s="7" t="n">
         <f aca="false">IF(F11="",E11,F11)*D11</f>
-        <v>517.5</v>
+        <v>288</v>
       </c>
       <c r="H11" s="25"/>
       <c r="I11" s="4"/>
@@ -1630,27 +1594,27 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B12" s="21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C12" s="22" t="str">
         <f aca="false">Riepilogo!$A$6</f>
-        <v>Elisa</v>
+        <v>Corina</v>
       </c>
       <c r="D12" s="23" t="n">
         <f aca="false">Riepilogo!$C$6</f>
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E12" s="24" t="n">
         <f aca="false">Riepilogo!$D$6*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B12,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B12+1,0))))</f>
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="F12" s="6"/>
       <c r="G12" s="7" t="n">
         <f aca="false">IF(F12="",E12,F12)*D12</f>
-        <v>360</v>
+        <v>160</v>
       </c>
       <c r="H12" s="25"/>
       <c r="I12" s="4"/>
@@ -1661,24 +1625,24 @@
         <v>69</v>
       </c>
       <c r="B13" s="21" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C13" s="22" t="str">
-        <f aca="false">Riepilogo!$A$7</f>
-        <v>Corina</v>
+        <f aca="false">Riepilogo!$A$5</f>
+        <v>Elisa</v>
       </c>
       <c r="D13" s="23" t="n">
-        <f aca="false">Riepilogo!$C$7</f>
-        <v>10</v>
+        <f aca="false">Riepilogo!$C$5</f>
+        <v>12</v>
       </c>
       <c r="E13" s="24" t="n">
-        <f aca="false">Riepilogo!$D$7*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B13,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B13+1,0))))</f>
-        <v>20</v>
+        <f aca="false">Riepilogo!$D$5*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B13,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B13+1,0))))</f>
+        <v>30</v>
       </c>
       <c r="F13" s="6"/>
       <c r="G13" s="7" t="n">
         <f aca="false">IF(F13="",E13,F13)*D13</f>
-        <v>200</v>
+        <v>360</v>
       </c>
       <c r="H13" s="25"/>
       <c r="I13" s="4"/>
@@ -1686,27 +1650,27 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B14" s="21" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C14" s="22" t="str">
-        <f aca="false">Riepilogo!$A$5</f>
-        <v>Oshina</v>
+        <f aca="false">Riepilogo!$A$6</f>
+        <v>Corina</v>
       </c>
       <c r="D14" s="23" t="n">
-        <f aca="false">Riepilogo!$C$5</f>
-        <v>11.5</v>
+        <f aca="false">Riepilogo!$C$6</f>
+        <v>10</v>
       </c>
       <c r="E14" s="24" t="n">
-        <f aca="false">Riepilogo!$D$5*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B14,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B14+1,0))))</f>
-        <v>36</v>
+        <f aca="false">Riepilogo!$D$6*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B14,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B14+1,0))))</f>
+        <v>20</v>
       </c>
       <c r="F14" s="6"/>
       <c r="G14" s="7" t="n">
         <f aca="false">IF(F14="",E14,F14)*D14</f>
-        <v>414</v>
+        <v>200</v>
       </c>
       <c r="H14" s="25"/>
       <c r="I14" s="4"/>
@@ -1717,18 +1681,18 @@
         <v>70</v>
       </c>
       <c r="B15" s="21" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C15" s="22" t="str">
-        <f aca="false">Riepilogo!$A$6</f>
+        <f aca="false">Riepilogo!$A$5</f>
         <v>Elisa</v>
       </c>
       <c r="D15" s="23" t="n">
-        <f aca="false">Riepilogo!$C$6</f>
+        <f aca="false">Riepilogo!$C$5</f>
         <v>12</v>
       </c>
       <c r="E15" s="24" t="n">
-        <f aca="false">Riepilogo!$D$6*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B15,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B15+1,0))))</f>
+        <f aca="false">Riepilogo!$D$5*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B15,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B15+1,0))))</f>
         <v>24</v>
       </c>
       <c r="F15" s="6"/>
@@ -1745,18 +1709,18 @@
         <v>70</v>
       </c>
       <c r="B16" s="21" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C16" s="22" t="str">
-        <f aca="false">Riepilogo!$A$7</f>
+        <f aca="false">Riepilogo!$A$6</f>
         <v>Corina</v>
       </c>
       <c r="D16" s="23" t="n">
-        <f aca="false">Riepilogo!$C$7</f>
+        <f aca="false">Riepilogo!$C$6</f>
         <v>10</v>
       </c>
       <c r="E16" s="24" t="n">
-        <f aca="false">Riepilogo!$D$7*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B16,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B16+1,0))))</f>
+        <f aca="false">Riepilogo!$D$6*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B16,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B16+1,0))))</f>
         <v>16</v>
       </c>
       <c r="F16" s="6"/>
@@ -1773,24 +1737,24 @@
         <v>71</v>
       </c>
       <c r="B17" s="21" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C17" s="22" t="str">
         <f aca="false">Riepilogo!$A$5</f>
-        <v>Oshina</v>
+        <v>Elisa</v>
       </c>
       <c r="D17" s="23" t="n">
         <f aca="false">Riepilogo!$C$5</f>
-        <v>11.5</v>
+        <v>12</v>
       </c>
       <c r="E17" s="24" t="n">
         <f aca="false">Riepilogo!$D$5*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B17,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B17+1,0))))</f>
-        <v>45</v>
+        <v>24</v>
       </c>
       <c r="F17" s="6"/>
       <c r="G17" s="7" t="n">
         <f aca="false">IF(F17="",E17,F17)*D17</f>
-        <v>517.5</v>
+        <v>288</v>
       </c>
       <c r="H17" s="25"/>
       <c r="I17" s="4"/>
@@ -1801,24 +1765,24 @@
         <v>71</v>
       </c>
       <c r="B18" s="21" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C18" s="22" t="str">
         <f aca="false">Riepilogo!$A$6</f>
-        <v>Elisa</v>
+        <v>Corina</v>
       </c>
       <c r="D18" s="23" t="n">
         <f aca="false">Riepilogo!$C$6</f>
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E18" s="24" t="n">
         <f aca="false">Riepilogo!$D$6*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B18,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B18+1,0))))</f>
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="F18" s="6"/>
       <c r="G18" s="7" t="n">
         <f aca="false">IF(F18="",E18,F18)*D18</f>
-        <v>360</v>
+        <v>160</v>
       </c>
       <c r="H18" s="25"/>
       <c r="I18" s="4"/>
@@ -1826,27 +1790,27 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="15" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B19" s="21" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C19" s="22" t="str">
-        <f aca="false">Riepilogo!$A$7</f>
-        <v>Corina</v>
+        <f aca="false">Riepilogo!$A$5</f>
+        <v>Elisa</v>
       </c>
       <c r="D19" s="23" t="n">
-        <f aca="false">Riepilogo!$C$7</f>
-        <v>10</v>
+        <f aca="false">Riepilogo!$C$5</f>
+        <v>12</v>
       </c>
       <c r="E19" s="24" t="n">
-        <f aca="false">Riepilogo!$D$7*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B19,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B19+1,0))))</f>
-        <v>20</v>
+        <f aca="false">Riepilogo!$D$5*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B19,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B19+1,0))))</f>
+        <v>30</v>
       </c>
       <c r="F19" s="6"/>
       <c r="G19" s="7" t="n">
         <f aca="false">IF(F19="",E19,F19)*D19</f>
-        <v>200</v>
+        <v>360</v>
       </c>
       <c r="H19" s="25"/>
       <c r="I19" s="4"/>
@@ -1857,24 +1821,24 @@
         <v>72</v>
       </c>
       <c r="B20" s="21" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C20" s="22" t="str">
-        <f aca="false">Riepilogo!$A$5</f>
-        <v>Oshina</v>
+        <f aca="false">Riepilogo!$A$6</f>
+        <v>Corina</v>
       </c>
       <c r="D20" s="23" t="n">
-        <f aca="false">Riepilogo!$C$5</f>
-        <v>11.5</v>
+        <f aca="false">Riepilogo!$C$6</f>
+        <v>10</v>
       </c>
       <c r="E20" s="24" t="n">
-        <f aca="false">Riepilogo!$D$5*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B20,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B20+1,0))))</f>
-        <v>36</v>
+        <f aca="false">Riepilogo!$D$6*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B20,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B20+1,0))))</f>
+        <v>20</v>
       </c>
       <c r="F20" s="6"/>
       <c r="G20" s="7" t="n">
         <f aca="false">IF(F20="",E20,F20)*D20</f>
-        <v>414</v>
+        <v>200</v>
       </c>
       <c r="H20" s="25"/>
       <c r="I20" s="4"/>
@@ -1882,21 +1846,21 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="15" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B21" s="21" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C21" s="22" t="str">
-        <f aca="false">Riepilogo!$A$6</f>
+        <f aca="false">Riepilogo!$A$5</f>
         <v>Elisa</v>
       </c>
       <c r="D21" s="23" t="n">
-        <f aca="false">Riepilogo!$C$6</f>
+        <f aca="false">Riepilogo!$C$5</f>
         <v>12</v>
       </c>
       <c r="E21" s="24" t="n">
-        <f aca="false">Riepilogo!$D$6*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B21,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B21+1,0))))</f>
+        <f aca="false">Riepilogo!$D$5*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B21,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B21+1,0))))</f>
         <v>24</v>
       </c>
       <c r="F21" s="6"/>
@@ -1910,21 +1874,21 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="15" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B22" s="21" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C22" s="22" t="str">
-        <f aca="false">Riepilogo!$A$7</f>
+        <f aca="false">Riepilogo!$A$6</f>
         <v>Corina</v>
       </c>
       <c r="D22" s="23" t="n">
-        <f aca="false">Riepilogo!$C$7</f>
+        <f aca="false">Riepilogo!$C$6</f>
         <v>10</v>
       </c>
       <c r="E22" s="24" t="n">
-        <f aca="false">Riepilogo!$D$7*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B22,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B22+1,0))))</f>
+        <f aca="false">Riepilogo!$D$6*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B22,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B22+1,0))))</f>
         <v>16</v>
       </c>
       <c r="F22" s="6"/>
@@ -1938,27 +1902,27 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="15" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B23" s="21" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C23" s="22" t="str">
         <f aca="false">Riepilogo!$A$5</f>
-        <v>Oshina</v>
+        <v>Elisa</v>
       </c>
       <c r="D23" s="23" t="n">
         <f aca="false">Riepilogo!$C$5</f>
-        <v>11.5</v>
+        <v>12</v>
       </c>
       <c r="E23" s="24" t="n">
         <f aca="false">Riepilogo!$D$5*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B23,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B23+1,0))))</f>
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="F23" s="6"/>
       <c r="G23" s="7" t="n">
         <f aca="false">IF(F23="",E23,F23)*D23</f>
-        <v>414</v>
+        <v>288</v>
       </c>
       <c r="H23" s="25"/>
       <c r="I23" s="4"/>
@@ -1966,27 +1930,27 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="15" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B24" s="21" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C24" s="22" t="str">
         <f aca="false">Riepilogo!$A$6</f>
-        <v>Elisa</v>
+        <v>Corina</v>
       </c>
       <c r="D24" s="23" t="n">
         <f aca="false">Riepilogo!$C$6</f>
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E24" s="24" t="n">
         <f aca="false">Riepilogo!$D$6*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B24,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B24+1,0))))</f>
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="F24" s="6"/>
       <c r="G24" s="7" t="n">
         <f aca="false">IF(F24="",E24,F24)*D24</f>
-        <v>288</v>
+        <v>160</v>
       </c>
       <c r="H24" s="25"/>
       <c r="I24" s="4"/>
@@ -1994,27 +1958,27 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="15" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B25" s="21" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="C25" s="22" t="str">
-        <f aca="false">Riepilogo!$A$7</f>
-        <v>Corina</v>
+        <f aca="false">Riepilogo!$A$5</f>
+        <v>Elisa</v>
       </c>
       <c r="D25" s="23" t="n">
-        <f aca="false">Riepilogo!$C$7</f>
-        <v>10</v>
+        <f aca="false">Riepilogo!$C$5</f>
+        <v>12</v>
       </c>
       <c r="E25" s="24" t="n">
-        <f aca="false">Riepilogo!$D$7*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B25,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B25+1,0))))</f>
-        <v>16</v>
+        <f aca="false">Riepilogo!$D$5*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B25,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B25+1,0))))</f>
+        <v>30</v>
       </c>
       <c r="F25" s="6"/>
       <c r="G25" s="7" t="n">
         <f aca="false">IF(F25="",E25,F25)*D25</f>
-        <v>160</v>
+        <v>360</v>
       </c>
       <c r="H25" s="25"/>
       <c r="I25" s="4"/>
@@ -2022,27 +1986,27 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="15" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B26" s="21" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C26" s="22" t="str">
-        <f aca="false">Riepilogo!$A$5</f>
-        <v>Oshina</v>
+        <f aca="false">Riepilogo!$A$6</f>
+        <v>Corina</v>
       </c>
       <c r="D26" s="23" t="n">
-        <f aca="false">Riepilogo!$C$5</f>
-        <v>11.5</v>
+        <f aca="false">Riepilogo!$C$6</f>
+        <v>10</v>
       </c>
       <c r="E26" s="24" t="n">
-        <f aca="false">Riepilogo!$D$5*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B26,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B26+1,0))))</f>
-        <v>45</v>
+        <f aca="false">Riepilogo!$D$6*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B26,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B26+1,0))))</f>
+        <v>20</v>
       </c>
       <c r="F26" s="6"/>
       <c r="G26" s="7" t="n">
         <f aca="false">IF(F26="",E26,F26)*D26</f>
-        <v>517.5</v>
+        <v>200</v>
       </c>
       <c r="H26" s="25"/>
       <c r="I26" s="4"/>
@@ -2050,27 +2014,27 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="15" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B27" s="21" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C27" s="22" t="str">
-        <f aca="false">Riepilogo!$A$6</f>
+        <f aca="false">Riepilogo!$A$5</f>
         <v>Elisa</v>
       </c>
       <c r="D27" s="23" t="n">
-        <f aca="false">Riepilogo!$C$6</f>
+        <f aca="false">Riepilogo!$C$5</f>
         <v>12</v>
       </c>
       <c r="E27" s="24" t="n">
-        <f aca="false">Riepilogo!$D$6*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B27,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B27+1,0))))</f>
-        <v>30</v>
+        <f aca="false">Riepilogo!$D$5*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B27,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B27+1,0))))</f>
+        <v>24</v>
       </c>
       <c r="F27" s="6"/>
       <c r="G27" s="7" t="n">
         <f aca="false">IF(F27="",E27,F27)*D27</f>
-        <v>360</v>
+        <v>288</v>
       </c>
       <c r="H27" s="25"/>
       <c r="I27" s="4"/>
@@ -2078,752 +2042,360 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="15" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B28" s="21" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C28" s="22" t="str">
-        <f aca="false">Riepilogo!$A$7</f>
+        <f aca="false">Riepilogo!$A$6</f>
         <v>Corina</v>
       </c>
       <c r="D28" s="23" t="n">
-        <f aca="false">Riepilogo!$C$7</f>
+        <f aca="false">Riepilogo!$C$6</f>
         <v>10</v>
       </c>
       <c r="E28" s="24" t="n">
-        <f aca="false">Riepilogo!$D$7*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B28,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B28+1,0))))</f>
-        <v>20</v>
+        <f aca="false">Riepilogo!$D$6*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B28,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B28+1,0))))</f>
+        <v>16</v>
       </c>
       <c r="F28" s="6"/>
       <c r="G28" s="7" t="n">
         <f aca="false">IF(F28="",E28,F28)*D28</f>
-        <v>200</v>
+        <v>160</v>
       </c>
       <c r="H28" s="25"/>
       <c r="I28" s="4"/>
       <c r="J28" s="26"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="15" t="s">
-        <v>75</v>
-      </c>
-      <c r="B29" s="21" t="n">
-        <v>9</v>
-      </c>
-      <c r="C29" s="22" t="str">
-        <f aca="false">Riepilogo!$A$5</f>
-        <v>Oshina</v>
-      </c>
-      <c r="D29" s="23" t="n">
-        <f aca="false">Riepilogo!$C$5</f>
-        <v>11.5</v>
-      </c>
-      <c r="E29" s="24" t="n">
-        <f aca="false">Riepilogo!$D$5*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B29,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B29+1,0))))</f>
-        <v>36</v>
-      </c>
-      <c r="F29" s="6"/>
-      <c r="G29" s="7" t="n">
-        <f aca="false">IF(F29="",E29,F29)*D29</f>
-        <v>414</v>
-      </c>
-      <c r="H29" s="25"/>
-      <c r="I29" s="4"/>
-      <c r="J29" s="26"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="15" t="s">
-        <v>75</v>
-      </c>
-      <c r="B30" s="21" t="n">
-        <v>9</v>
-      </c>
-      <c r="C30" s="22" t="str">
-        <f aca="false">Riepilogo!$A$6</f>
+      <c r="A29" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="B29" s="10"/>
+      <c r="C29" s="10"/>
+      <c r="D29" s="10"/>
+      <c r="E29" s="12" t="n">
+        <f aca="false">SUM(E5:E28)</f>
+        <v>520</v>
+      </c>
+      <c r="F29" s="12" t="n">
+        <f aca="false">SUM(F5:F28)</f>
+        <v>0</v>
+      </c>
+      <c r="G29" s="11" t="n">
+        <f aca="false">SUM(G5:G28)</f>
+        <v>5824</v>
+      </c>
+      <c r="H29" s="10"/>
+      <c r="I29" s="10"/>
+      <c r="J29" s="10"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="14" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B33" s="3" t="str">
+        <f aca="false">Riepilogo!A5</f>
         <v>Elisa</v>
       </c>
-      <c r="D30" s="23" t="n">
-        <f aca="false">Riepilogo!$C$6</f>
-        <v>12</v>
-      </c>
-      <c r="E30" s="24" t="n">
-        <f aca="false">Riepilogo!$D$6*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B30,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B30+1,0))))</f>
-        <v>24</v>
-      </c>
-      <c r="F30" s="6"/>
-      <c r="G30" s="7" t="n">
-        <f aca="false">IF(F30="",E30,F30)*D30</f>
-        <v>288</v>
-      </c>
-      <c r="H30" s="25"/>
-      <c r="I30" s="4"/>
-      <c r="J30" s="26"/>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="15" t="s">
-        <v>75</v>
-      </c>
-      <c r="B31" s="21" t="n">
-        <v>9</v>
-      </c>
-      <c r="C31" s="22" t="str">
-        <f aca="false">Riepilogo!$A$7</f>
+      <c r="C33" s="3" t="str">
+        <f aca="false">Riepilogo!A6</f>
         <v>Corina</v>
       </c>
-      <c r="D31" s="23" t="n">
-        <f aca="false">Riepilogo!$C$7</f>
-        <v>10</v>
-      </c>
-      <c r="E31" s="24" t="n">
-        <f aca="false">Riepilogo!$D$7*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B31,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B31+1,0))))</f>
-        <v>16</v>
-      </c>
-      <c r="F31" s="6"/>
-      <c r="G31" s="7" t="n">
-        <f aca="false">IF(F31="",E31,F31)*D31</f>
-        <v>160</v>
-      </c>
-      <c r="H31" s="25"/>
-      <c r="I31" s="4"/>
-      <c r="J31" s="26"/>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="15" t="s">
-        <v>76</v>
-      </c>
-      <c r="B32" s="21" t="n">
-        <v>10</v>
-      </c>
-      <c r="C32" s="22" t="str">
-        <f aca="false">Riepilogo!$A$5</f>
-        <v>Oshina</v>
-      </c>
-      <c r="D32" s="23" t="n">
-        <f aca="false">Riepilogo!$C$5</f>
-        <v>11.5</v>
-      </c>
-      <c r="E32" s="24" t="n">
-        <f aca="false">Riepilogo!$D$5*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B32,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B32+1,0))))</f>
-        <v>36</v>
-      </c>
-      <c r="F32" s="6"/>
-      <c r="G32" s="7" t="n">
-        <f aca="false">IF(F32="",E32,F32)*D32</f>
-        <v>414</v>
-      </c>
-      <c r="H32" s="25"/>
-      <c r="I32" s="4"/>
-      <c r="J32" s="26"/>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="15" t="s">
-        <v>76</v>
-      </c>
-      <c r="B33" s="21" t="n">
-        <v>10</v>
-      </c>
-      <c r="C33" s="22" t="str">
-        <f aca="false">Riepilogo!$A$6</f>
-        <v>Elisa</v>
-      </c>
-      <c r="D33" s="23" t="n">
-        <f aca="false">Riepilogo!$C$6</f>
-        <v>12</v>
-      </c>
-      <c r="E33" s="24" t="n">
-        <f aca="false">Riepilogo!$D$6*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B33,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B33+1,0))))</f>
-        <v>24</v>
-      </c>
-      <c r="F33" s="6"/>
-      <c r="G33" s="7" t="n">
-        <f aca="false">IF(F33="",E33,F33)*D33</f>
-        <v>288</v>
-      </c>
-      <c r="H33" s="25"/>
-      <c r="I33" s="4"/>
-      <c r="J33" s="26"/>
+      <c r="D33" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="15" t="s">
-        <v>76</v>
-      </c>
-      <c r="B34" s="21" t="n">
-        <v>10</v>
-      </c>
-      <c r="C34" s="22" t="str">
-        <f aca="false">Riepilogo!$A$7</f>
-        <v>Corina</v>
-      </c>
-      <c r="D34" s="23" t="n">
-        <f aca="false">Riepilogo!$C$7</f>
-        <v>10</v>
-      </c>
-      <c r="E34" s="24" t="n">
-        <f aca="false">Riepilogo!$D$7*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B34,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B34+1,0))))</f>
-        <v>16</v>
-      </c>
-      <c r="F34" s="6"/>
-      <c r="G34" s="7" t="n">
-        <f aca="false">IF(F34="",E34,F34)*D34</f>
+        <v>65</v>
+      </c>
+      <c r="B34" s="7" t="n">
+        <f aca="false">SUMIFS($G$5:$G$28,$B$5:$B$28,1,$C$5:$C$28,B$33)</f>
+        <v>288</v>
+      </c>
+      <c r="C34" s="7" t="n">
+        <f aca="false">SUMIFS($G$5:$G$28,$B$5:$B$28,1,$C$5:$C$28,C$33)</f>
         <v>160</v>
       </c>
-      <c r="H34" s="25"/>
-      <c r="I34" s="4"/>
-      <c r="J34" s="26"/>
+      <c r="D34" s="8" t="n">
+        <f aca="false">SUM(B34:C34)</f>
+        <v>448</v>
+      </c>
+      <c r="E34" s="21" t="n">
+        <f aca="false">COUNTIFS($B$5:$B$28,1,$I$5:$I$28,"&lt;&gt;SI")</f>
+        <v>2</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="15" t="s">
-        <v>77</v>
-      </c>
-      <c r="B35" s="21" t="n">
-        <v>11</v>
-      </c>
-      <c r="C35" s="22" t="str">
-        <f aca="false">Riepilogo!$A$5</f>
-        <v>Oshina</v>
-      </c>
-      <c r="D35" s="23" t="n">
-        <f aca="false">Riepilogo!$C$5</f>
-        <v>11.5</v>
-      </c>
-      <c r="E35" s="24" t="n">
-        <f aca="false">Riepilogo!$D$5*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B35,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B35+1,0))))</f>
-        <v>45</v>
-      </c>
-      <c r="F35" s="6"/>
-      <c r="G35" s="7" t="n">
-        <f aca="false">IF(F35="",E35,F35)*D35</f>
-        <v>517.5</v>
-      </c>
-      <c r="H35" s="25"/>
-      <c r="I35" s="4"/>
-      <c r="J35" s="26"/>
+        <v>66</v>
+      </c>
+      <c r="B35" s="7" t="n">
+        <f aca="false">SUMIFS($G$5:$G$28,$B$5:$B$28,2,$C$5:$C$28,B$33)</f>
+        <v>288</v>
+      </c>
+      <c r="C35" s="7" t="n">
+        <f aca="false">SUMIFS($G$5:$G$28,$B$5:$B$28,2,$C$5:$C$28,C$33)</f>
+        <v>160</v>
+      </c>
+      <c r="D35" s="8" t="n">
+        <f aca="false">SUM(B35:C35)</f>
+        <v>448</v>
+      </c>
+      <c r="E35" s="21" t="n">
+        <f aca="false">COUNTIFS($B$5:$B$28,2,$I$5:$I$28,"&lt;&gt;SI")</f>
+        <v>2</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="15" t="s">
-        <v>77</v>
-      </c>
-      <c r="B36" s="21" t="n">
-        <v>11</v>
-      </c>
-      <c r="C36" s="22" t="str">
-        <f aca="false">Riepilogo!$A$6</f>
-        <v>Elisa</v>
-      </c>
-      <c r="D36" s="23" t="n">
-        <f aca="false">Riepilogo!$C$6</f>
-        <v>12</v>
-      </c>
-      <c r="E36" s="24" t="n">
-        <f aca="false">Riepilogo!$D$6*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B36,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B36+1,0))))</f>
-        <v>30</v>
-      </c>
-      <c r="F36" s="6"/>
-      <c r="G36" s="7" t="n">
-        <f aca="false">IF(F36="",E36,F36)*D36</f>
+        <v>67</v>
+      </c>
+      <c r="B36" s="7" t="n">
+        <f aca="false">SUMIFS($G$5:$G$28,$B$5:$B$28,3,$C$5:$C$28,B$33)</f>
         <v>360</v>
       </c>
-      <c r="H36" s="25"/>
-      <c r="I36" s="4"/>
-      <c r="J36" s="26"/>
+      <c r="C36" s="7" t="n">
+        <f aca="false">SUMIFS($G$5:$G$28,$B$5:$B$28,3,$C$5:$C$28,C$33)</f>
+        <v>200</v>
+      </c>
+      <c r="D36" s="8" t="n">
+        <f aca="false">SUM(B36:C36)</f>
+        <v>560</v>
+      </c>
+      <c r="E36" s="21" t="n">
+        <f aca="false">COUNTIFS($B$5:$B$28,3,$I$5:$I$28,"&lt;&gt;SI")</f>
+        <v>2</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="15" t="s">
-        <v>77</v>
-      </c>
-      <c r="B37" s="21" t="n">
-        <v>11</v>
-      </c>
-      <c r="C37" s="22" t="str">
-        <f aca="false">Riepilogo!$A$7</f>
-        <v>Corina</v>
-      </c>
-      <c r="D37" s="23" t="n">
-        <f aca="false">Riepilogo!$C$7</f>
-        <v>10</v>
-      </c>
-      <c r="E37" s="24" t="n">
-        <f aca="false">Riepilogo!$D$7*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B37,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B37+1,0))))</f>
-        <v>20</v>
-      </c>
-      <c r="F37" s="6"/>
-      <c r="G37" s="7" t="n">
-        <f aca="false">IF(F37="",E37,F37)*D37</f>
-        <v>200</v>
-      </c>
-      <c r="H37" s="25"/>
-      <c r="I37" s="4"/>
-      <c r="J37" s="26"/>
+        <v>68</v>
+      </c>
+      <c r="B37" s="7" t="n">
+        <f aca="false">SUMIFS($G$5:$G$28,$B$5:$B$28,4,$C$5:$C$28,B$33)</f>
+        <v>288</v>
+      </c>
+      <c r="C37" s="7" t="n">
+        <f aca="false">SUMIFS($G$5:$G$28,$B$5:$B$28,4,$C$5:$C$28,C$33)</f>
+        <v>160</v>
+      </c>
+      <c r="D37" s="8" t="n">
+        <f aca="false">SUM(B37:C37)</f>
+        <v>448</v>
+      </c>
+      <c r="E37" s="21" t="n">
+        <f aca="false">COUNTIFS($B$5:$B$28,4,$I$5:$I$28,"&lt;&gt;SI")</f>
+        <v>2</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="15" t="s">
-        <v>78</v>
-      </c>
-      <c r="B38" s="21" t="n">
-        <v>12</v>
-      </c>
-      <c r="C38" s="22" t="str">
-        <f aca="false">Riepilogo!$A$5</f>
-        <v>Oshina</v>
-      </c>
-      <c r="D38" s="23" t="n">
-        <f aca="false">Riepilogo!$C$5</f>
-        <v>11.5</v>
-      </c>
-      <c r="E38" s="24" t="n">
-        <f aca="false">Riepilogo!$D$5*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B38,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B38+1,0))))</f>
-        <v>36</v>
-      </c>
-      <c r="F38" s="6"/>
-      <c r="G38" s="7" t="n">
-        <f aca="false">IF(F38="",E38,F38)*D38</f>
-        <v>414</v>
-      </c>
-      <c r="H38" s="25"/>
-      <c r="I38" s="4"/>
-      <c r="J38" s="26"/>
+        <v>69</v>
+      </c>
+      <c r="B38" s="7" t="n">
+        <f aca="false">SUMIFS($G$5:$G$28,$B$5:$B$28,5,$C$5:$C$28,B$33)</f>
+        <v>360</v>
+      </c>
+      <c r="C38" s="7" t="n">
+        <f aca="false">SUMIFS($G$5:$G$28,$B$5:$B$28,5,$C$5:$C$28,C$33)</f>
+        <v>200</v>
+      </c>
+      <c r="D38" s="8" t="n">
+        <f aca="false">SUM(B38:C38)</f>
+        <v>560</v>
+      </c>
+      <c r="E38" s="21" t="n">
+        <f aca="false">COUNTIFS($B$5:$B$28,5,$I$5:$I$28,"&lt;&gt;SI")</f>
+        <v>2</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="15" t="s">
-        <v>78</v>
-      </c>
-      <c r="B39" s="21" t="n">
-        <v>12</v>
-      </c>
-      <c r="C39" s="22" t="str">
-        <f aca="false">Riepilogo!$A$6</f>
-        <v>Elisa</v>
-      </c>
-      <c r="D39" s="23" t="n">
-        <f aca="false">Riepilogo!$C$6</f>
-        <v>12</v>
-      </c>
-      <c r="E39" s="24" t="n">
-        <f aca="false">Riepilogo!$D$6*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B39,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B39+1,0))))</f>
-        <v>24</v>
-      </c>
-      <c r="F39" s="6"/>
-      <c r="G39" s="7" t="n">
-        <f aca="false">IF(F39="",E39,F39)*D39</f>
+        <v>70</v>
+      </c>
+      <c r="B39" s="7" t="n">
+        <f aca="false">SUMIFS($G$5:$G$28,$B$5:$B$28,6,$C$5:$C$28,B$33)</f>
         <v>288</v>
       </c>
-      <c r="H39" s="25"/>
-      <c r="I39" s="4"/>
-      <c r="J39" s="26"/>
+      <c r="C39" s="7" t="n">
+        <f aca="false">SUMIFS($G$5:$G$28,$B$5:$B$28,6,$C$5:$C$28,C$33)</f>
+        <v>160</v>
+      </c>
+      <c r="D39" s="8" t="n">
+        <f aca="false">SUM(B39:C39)</f>
+        <v>448</v>
+      </c>
+      <c r="E39" s="21" t="n">
+        <f aca="false">COUNTIFS($B$5:$B$28,6,$I$5:$I$28,"&lt;&gt;SI")</f>
+        <v>2</v>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="15" t="s">
-        <v>78</v>
-      </c>
-      <c r="B40" s="21" t="n">
-        <v>12</v>
-      </c>
-      <c r="C40" s="22" t="str">
-        <f aca="false">Riepilogo!$A$7</f>
-        <v>Corina</v>
-      </c>
-      <c r="D40" s="23" t="n">
-        <f aca="false">Riepilogo!$C$7</f>
-        <v>10</v>
-      </c>
-      <c r="E40" s="24" t="n">
-        <f aca="false">Riepilogo!$D$7*SUMPRODUCT(--(WEEKDAY(DATE(Parametri!$B$5,B40,1)+ROW($A$1:$A$31)-1,2)=1),--(ROW($A$1:$A$31)&lt;=DAY(DATE(Parametri!$B$5,B40+1,0))))</f>
-        <v>16</v>
-      </c>
-      <c r="F40" s="6"/>
-      <c r="G40" s="7" t="n">
-        <f aca="false">IF(F40="",E40,F40)*D40</f>
+        <v>71</v>
+      </c>
+      <c r="B40" s="7" t="n">
+        <f aca="false">SUMIFS($G$5:$G$28,$B$5:$B$28,7,$C$5:$C$28,B$33)</f>
+        <v>288</v>
+      </c>
+      <c r="C40" s="7" t="n">
+        <f aca="false">SUMIFS($G$5:$G$28,$B$5:$B$28,7,$C$5:$C$28,C$33)</f>
         <v>160</v>
       </c>
-      <c r="H40" s="25"/>
-      <c r="I40" s="4"/>
-      <c r="J40" s="26"/>
+      <c r="D40" s="8" t="n">
+        <f aca="false">SUM(B40:C40)</f>
+        <v>448</v>
+      </c>
+      <c r="E40" s="21" t="n">
+        <f aca="false">COUNTIFS($B$5:$B$28,7,$I$5:$I$28,"&lt;&gt;SI")</f>
+        <v>2</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="B41" s="10"/>
-      <c r="C41" s="10"/>
-      <c r="D41" s="10"/>
-      <c r="E41" s="12" t="n">
-        <f aca="false">SUM(E5:E40)</f>
-        <v>988</v>
-      </c>
-      <c r="F41" s="12" t="n">
-        <f aca="false">SUM(F5:F40)</f>
-        <v>0</v>
-      </c>
-      <c r="G41" s="11" t="n">
-        <f aca="false">SUM(G5:G40)</f>
-        <v>11206</v>
-      </c>
-      <c r="H41" s="10"/>
-      <c r="I41" s="10"/>
-      <c r="J41" s="10"/>
+      <c r="A41" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="B41" s="7" t="n">
+        <f aca="false">SUMIFS($G$5:$G$28,$B$5:$B$28,8,$C$5:$C$28,B$33)</f>
+        <v>360</v>
+      </c>
+      <c r="C41" s="7" t="n">
+        <f aca="false">SUMIFS($G$5:$G$28,$B$5:$B$28,8,$C$5:$C$28,C$33)</f>
+        <v>200</v>
+      </c>
+      <c r="D41" s="8" t="n">
+        <f aca="false">SUM(B41:C41)</f>
+        <v>560</v>
+      </c>
+      <c r="E41" s="21" t="n">
+        <f aca="false">COUNTIFS($B$5:$B$28,8,$I$5:$I$28,"&lt;&gt;SI")</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="B42" s="7" t="n">
+        <f aca="false">SUMIFS($G$5:$G$28,$B$5:$B$28,9,$C$5:$C$28,B$33)</f>
+        <v>288</v>
+      </c>
+      <c r="C42" s="7" t="n">
+        <f aca="false">SUMIFS($G$5:$G$28,$B$5:$B$28,9,$C$5:$C$28,C$33)</f>
+        <v>160</v>
+      </c>
+      <c r="D42" s="8" t="n">
+        <f aca="false">SUM(B42:C42)</f>
+        <v>448</v>
+      </c>
+      <c r="E42" s="21" t="n">
+        <f aca="false">COUNTIFS($B$5:$B$28,9,$I$5:$I$28,"&lt;&gt;SI")</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="B43" s="7" t="n">
+        <f aca="false">SUMIFS($G$5:$G$28,$B$5:$B$28,10,$C$5:$C$28,B$33)</f>
+        <v>288</v>
+      </c>
+      <c r="C43" s="7" t="n">
+        <f aca="false">SUMIFS($G$5:$G$28,$B$5:$B$28,10,$C$5:$C$28,C$33)</f>
+        <v>160</v>
+      </c>
+      <c r="D43" s="8" t="n">
+        <f aca="false">SUM(B43:C43)</f>
+        <v>448</v>
+      </c>
+      <c r="E43" s="21" t="n">
+        <f aca="false">COUNTIFS($B$5:$B$28,10,$I$5:$I$28,"&lt;&gt;SI")</f>
+        <v>2</v>
+      </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="14" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="B45" s="3" t="str">
-        <f aca="false">Riepilogo!A5</f>
-        <v>Oshina</v>
-      </c>
-      <c r="C45" s="3" t="str">
-        <f aca="false">Riepilogo!A6</f>
-        <v>Elisa</v>
-      </c>
-      <c r="D45" s="3" t="str">
-        <f aca="false">Riepilogo!A7</f>
-        <v>Corina</v>
-      </c>
-      <c r="E45" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="F45" s="3" t="s">
-        <v>82</v>
+      <c r="A44" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="B44" s="7" t="n">
+        <f aca="false">SUMIFS($G$5:$G$28,$B$5:$B$28,11,$C$5:$C$28,B$33)</f>
+        <v>360</v>
+      </c>
+      <c r="C44" s="7" t="n">
+        <f aca="false">SUMIFS($G$5:$G$28,$B$5:$B$28,11,$C$5:$C$28,C$33)</f>
+        <v>200</v>
+      </c>
+      <c r="D44" s="8" t="n">
+        <f aca="false">SUM(B44:C44)</f>
+        <v>560</v>
+      </c>
+      <c r="E44" s="21" t="n">
+        <f aca="false">COUNTIFS($B$5:$B$28,11,$I$5:$I$28,"&lt;&gt;SI")</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="B45" s="7" t="n">
+        <f aca="false">SUMIFS($G$5:$G$28,$B$5:$B$28,12,$C$5:$C$28,B$33)</f>
+        <v>288</v>
+      </c>
+      <c r="C45" s="7" t="n">
+        <f aca="false">SUMIFS($G$5:$G$28,$B$5:$B$28,12,$C$5:$C$28,C$33)</f>
+        <v>160</v>
+      </c>
+      <c r="D45" s="8" t="n">
+        <f aca="false">SUM(B45:C45)</f>
+        <v>448</v>
+      </c>
+      <c r="E45" s="21" t="n">
+        <f aca="false">COUNTIFS($B$5:$B$28,12,$I$5:$I$28,"&lt;&gt;SI")</f>
+        <v>2</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="15" t="s">
-        <v>67</v>
-      </c>
-      <c r="B46" s="7" t="n">
-        <f aca="false">SUMIFS($G$5:$G$40,$B$5:$B$40,1,$C$5:$C$40,B$45)</f>
-        <v>414</v>
-      </c>
-      <c r="C46" s="7" t="n">
-        <f aca="false">SUMIFS($G$5:$G$40,$B$5:$B$40,1,$C$5:$C$40,C$45)</f>
-        <v>288</v>
-      </c>
-      <c r="D46" s="7" t="n">
-        <f aca="false">SUMIFS($G$5:$G$40,$B$5:$B$40,1,$C$5:$C$40,D$45)</f>
-        <v>160</v>
-      </c>
-      <c r="E46" s="8" t="n">
-        <f aca="false">SUM(B46:D46)</f>
-        <v>862</v>
-      </c>
-      <c r="F46" s="21" t="n">
-        <f aca="false">COUNTIFS($B$5:$B$40,1,$I$5:$I$40,"&lt;&gt;SI")</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="15" t="s">
-        <v>68</v>
-      </c>
-      <c r="B47" s="7" t="n">
-        <f aca="false">SUMIFS($G$5:$G$40,$B$5:$B$40,2,$C$5:$C$40,B$45)</f>
-        <v>414</v>
-      </c>
-      <c r="C47" s="7" t="n">
-        <f aca="false">SUMIFS($G$5:$G$40,$B$5:$B$40,2,$C$5:$C$40,C$45)</f>
-        <v>288</v>
-      </c>
-      <c r="D47" s="7" t="n">
-        <f aca="false">SUMIFS($G$5:$G$40,$B$5:$B$40,2,$C$5:$C$40,D$45)</f>
-        <v>160</v>
-      </c>
-      <c r="E47" s="8" t="n">
-        <f aca="false">SUM(B47:D47)</f>
-        <v>862</v>
-      </c>
-      <c r="F47" s="21" t="n">
-        <f aca="false">COUNTIFS($B$5:$B$40,2,$I$5:$I$40,"&lt;&gt;SI")</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="15" t="s">
-        <v>69</v>
-      </c>
-      <c r="B48" s="7" t="n">
-        <f aca="false">SUMIFS($G$5:$G$40,$B$5:$B$40,3,$C$5:$C$40,B$45)</f>
-        <v>517.5</v>
-      </c>
-      <c r="C48" s="7" t="n">
-        <f aca="false">SUMIFS($G$5:$G$40,$B$5:$B$40,3,$C$5:$C$40,C$45)</f>
-        <v>360</v>
-      </c>
-      <c r="D48" s="7" t="n">
-        <f aca="false">SUMIFS($G$5:$G$40,$B$5:$B$40,3,$C$5:$C$40,D$45)</f>
-        <v>200</v>
-      </c>
-      <c r="E48" s="8" t="n">
-        <f aca="false">SUM(B48:D48)</f>
-        <v>1077.5</v>
-      </c>
-      <c r="F48" s="21" t="n">
-        <f aca="false">COUNTIFS($B$5:$B$40,3,$I$5:$I$40,"&lt;&gt;SI")</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="B49" s="7" t="n">
-        <f aca="false">SUMIFS($G$5:$G$40,$B$5:$B$40,4,$C$5:$C$40,B$45)</f>
-        <v>414</v>
-      </c>
-      <c r="C49" s="7" t="n">
-        <f aca="false">SUMIFS($G$5:$G$40,$B$5:$B$40,4,$C$5:$C$40,C$45)</f>
-        <v>288</v>
-      </c>
-      <c r="D49" s="7" t="n">
-        <f aca="false">SUMIFS($G$5:$G$40,$B$5:$B$40,4,$C$5:$C$40,D$45)</f>
-        <v>160</v>
-      </c>
-      <c r="E49" s="8" t="n">
-        <f aca="false">SUM(B49:D49)</f>
-        <v>862</v>
-      </c>
-      <c r="F49" s="21" t="n">
-        <f aca="false">COUNTIFS($B$5:$B$40,4,$I$5:$I$40,"&lt;&gt;SI")</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="15" t="s">
-        <v>71</v>
-      </c>
-      <c r="B50" s="7" t="n">
-        <f aca="false">SUMIFS($G$5:$G$40,$B$5:$B$40,5,$C$5:$C$40,B$45)</f>
-        <v>517.5</v>
-      </c>
-      <c r="C50" s="7" t="n">
-        <f aca="false">SUMIFS($G$5:$G$40,$B$5:$B$40,5,$C$5:$C$40,C$45)</f>
-        <v>360</v>
-      </c>
-      <c r="D50" s="7" t="n">
-        <f aca="false">SUMIFS($G$5:$G$40,$B$5:$B$40,5,$C$5:$C$40,D$45)</f>
-        <v>200</v>
-      </c>
-      <c r="E50" s="8" t="n">
-        <f aca="false">SUM(B50:D50)</f>
-        <v>1077.5</v>
-      </c>
-      <c r="F50" s="21" t="n">
-        <f aca="false">COUNTIFS($B$5:$B$40,5,$I$5:$I$40,"&lt;&gt;SI")</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="B51" s="7" t="n">
-        <f aca="false">SUMIFS($G$5:$G$40,$B$5:$B$40,6,$C$5:$C$40,B$45)</f>
-        <v>414</v>
-      </c>
-      <c r="C51" s="7" t="n">
-        <f aca="false">SUMIFS($G$5:$G$40,$B$5:$B$40,6,$C$5:$C$40,C$45)</f>
-        <v>288</v>
-      </c>
-      <c r="D51" s="7" t="n">
-        <f aca="false">SUMIFS($G$5:$G$40,$B$5:$B$40,6,$C$5:$C$40,D$45)</f>
-        <v>160</v>
-      </c>
-      <c r="E51" s="8" t="n">
-        <f aca="false">SUM(B51:D51)</f>
-        <v>862</v>
-      </c>
-      <c r="F51" s="21" t="n">
-        <f aca="false">COUNTIFS($B$5:$B$40,6,$I$5:$I$40,"&lt;&gt;SI")</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="15" t="s">
-        <v>73</v>
-      </c>
-      <c r="B52" s="7" t="n">
-        <f aca="false">SUMIFS($G$5:$G$40,$B$5:$B$40,7,$C$5:$C$40,B$45)</f>
-        <v>414</v>
-      </c>
-      <c r="C52" s="7" t="n">
-        <f aca="false">SUMIFS($G$5:$G$40,$B$5:$B$40,7,$C$5:$C$40,C$45)</f>
-        <v>288</v>
-      </c>
-      <c r="D52" s="7" t="n">
-        <f aca="false">SUMIFS($G$5:$G$40,$B$5:$B$40,7,$C$5:$C$40,D$45)</f>
-        <v>160</v>
-      </c>
-      <c r="E52" s="8" t="n">
-        <f aca="false">SUM(B52:D52)</f>
-        <v>862</v>
-      </c>
-      <c r="F52" s="21" t="n">
-        <f aca="false">COUNTIFS($B$5:$B$40,7,$I$5:$I$40,"&lt;&gt;SI")</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="15" t="s">
-        <v>74</v>
-      </c>
-      <c r="B53" s="7" t="n">
-        <f aca="false">SUMIFS($G$5:$G$40,$B$5:$B$40,8,$C$5:$C$40,B$45)</f>
-        <v>517.5</v>
-      </c>
-      <c r="C53" s="7" t="n">
-        <f aca="false">SUMIFS($G$5:$G$40,$B$5:$B$40,8,$C$5:$C$40,C$45)</f>
-        <v>360</v>
-      </c>
-      <c r="D53" s="7" t="n">
-        <f aca="false">SUMIFS($G$5:$G$40,$B$5:$B$40,8,$C$5:$C$40,D$45)</f>
-        <v>200</v>
-      </c>
-      <c r="E53" s="8" t="n">
-        <f aca="false">SUM(B53:D53)</f>
-        <v>1077.5</v>
-      </c>
-      <c r="F53" s="21" t="n">
-        <f aca="false">COUNTIFS($B$5:$B$40,8,$I$5:$I$40,"&lt;&gt;SI")</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="15" t="s">
-        <v>75</v>
-      </c>
-      <c r="B54" s="7" t="n">
-        <f aca="false">SUMIFS($G$5:$G$40,$B$5:$B$40,9,$C$5:$C$40,B$45)</f>
-        <v>414</v>
-      </c>
-      <c r="C54" s="7" t="n">
-        <f aca="false">SUMIFS($G$5:$G$40,$B$5:$B$40,9,$C$5:$C$40,C$45)</f>
-        <v>288</v>
-      </c>
-      <c r="D54" s="7" t="n">
-        <f aca="false">SUMIFS($G$5:$G$40,$B$5:$B$40,9,$C$5:$C$40,D$45)</f>
-        <v>160</v>
-      </c>
-      <c r="E54" s="8" t="n">
-        <f aca="false">SUM(B54:D54)</f>
-        <v>862</v>
-      </c>
-      <c r="F54" s="21" t="n">
-        <f aca="false">COUNTIFS($B$5:$B$40,9,$I$5:$I$40,"&lt;&gt;SI")</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="15" t="s">
-        <v>76</v>
-      </c>
-      <c r="B55" s="7" t="n">
-        <f aca="false">SUMIFS($G$5:$G$40,$B$5:$B$40,10,$C$5:$C$40,B$45)</f>
-        <v>414</v>
-      </c>
-      <c r="C55" s="7" t="n">
-        <f aca="false">SUMIFS($G$5:$G$40,$B$5:$B$40,10,$C$5:$C$40,C$45)</f>
-        <v>288</v>
-      </c>
-      <c r="D55" s="7" t="n">
-        <f aca="false">SUMIFS($G$5:$G$40,$B$5:$B$40,10,$C$5:$C$40,D$45)</f>
-        <v>160</v>
-      </c>
-      <c r="E55" s="8" t="n">
-        <f aca="false">SUM(B55:D55)</f>
-        <v>862</v>
-      </c>
-      <c r="F55" s="21" t="n">
-        <f aca="false">COUNTIFS($B$5:$B$40,10,$I$5:$I$40,"&lt;&gt;SI")</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="15" t="s">
-        <v>77</v>
-      </c>
-      <c r="B56" s="7" t="n">
-        <f aca="false">SUMIFS($G$5:$G$40,$B$5:$B$40,11,$C$5:$C$40,B$45)</f>
-        <v>517.5</v>
-      </c>
-      <c r="C56" s="7" t="n">
-        <f aca="false">SUMIFS($G$5:$G$40,$B$5:$B$40,11,$C$5:$C$40,C$45)</f>
-        <v>360</v>
-      </c>
-      <c r="D56" s="7" t="n">
-        <f aca="false">SUMIFS($G$5:$G$40,$B$5:$B$40,11,$C$5:$C$40,D$45)</f>
-        <v>200</v>
-      </c>
-      <c r="E56" s="8" t="n">
-        <f aca="false">SUM(B56:D56)</f>
-        <v>1077.5</v>
-      </c>
-      <c r="F56" s="21" t="n">
-        <f aca="false">COUNTIFS($B$5:$B$40,11,$I$5:$I$40,"&lt;&gt;SI")</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="15" t="s">
-        <v>78</v>
-      </c>
-      <c r="B57" s="7" t="n">
-        <f aca="false">SUMIFS($G$5:$G$40,$B$5:$B$40,12,$C$5:$C$40,B$45)</f>
-        <v>414</v>
-      </c>
-      <c r="C57" s="7" t="n">
-        <f aca="false">SUMIFS($G$5:$G$40,$B$5:$B$40,12,$C$5:$C$40,C$45)</f>
-        <v>288</v>
-      </c>
-      <c r="D57" s="7" t="n">
-        <f aca="false">SUMIFS($G$5:$G$40,$B$5:$B$40,12,$C$5:$C$40,D$45)</f>
-        <v>160</v>
-      </c>
-      <c r="E57" s="8" t="n">
-        <f aca="false">SUM(B57:D57)</f>
-        <v>862</v>
-      </c>
-      <c r="F57" s="21" t="n">
-        <f aca="false">COUNTIFS($B$5:$B$40,12,$I$5:$I$40,"&lt;&gt;SI")</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="B58" s="11" t="n">
-        <f aca="false">SUM(B46:B57)</f>
-        <v>5382</v>
-      </c>
-      <c r="C58" s="11" t="n">
-        <f aca="false">SUM(C46:C57)</f>
+      <c r="A46" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B46" s="11" t="n">
+        <f aca="false">SUM(B34:B45)</f>
         <v>3744</v>
       </c>
-      <c r="D58" s="11" t="n">
-        <f aca="false">SUM(D46:D57)</f>
+      <c r="C46" s="11" t="n">
+        <f aca="false">SUM(C34:C45)</f>
         <v>2080</v>
       </c>
-      <c r="E58" s="11" t="n">
-        <f aca="false">SUM(E46:E57)</f>
-        <v>11206</v>
-      </c>
-      <c r="F58" s="27" t="n">
-        <f aca="false">SUM(F46:F57)</f>
-        <v>36</v>
+      <c r="D46" s="11" t="n">
+        <f aca="false">SUM(D34:D45)</f>
+        <v>5824</v>
+      </c>
+      <c r="E46" s="27" t="n">
+        <f aca="false">SUM(E34:E45)</f>
+        <v>24</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I5:I40">
+  <conditionalFormatting sqref="I5:I28">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>"NO"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I5:I40" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I5:I28" type="list">
       <formula1>"SI,NO"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2843,7 +2415,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M23"/>
+  <dimension ref="A1:M22"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
@@ -2857,12 +2429,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2870,58 +2442,58 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="F4" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="G4" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="H4" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="I4" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="J4" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="K4" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="J4" s="3" t="s">
+      <c r="L4" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="K4" s="3" t="s">
+      <c r="M4" s="3" t="s">
         <v>94</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="M4" s="3" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="22" t="str">
         <f aca="false">Riepilogo!A5</f>
-        <v>Oshina</v>
+        <v>Elisa</v>
       </c>
       <c r="B5" s="7" t="n">
         <f aca="false">Riepilogo!E5*Parametri!$B$12</f>
-        <v>5382</v>
+        <v>3744</v>
       </c>
       <c r="C5" s="7" t="n">
         <f aca="false">B5/Parametri!$B$7*Parametri!$B$13</f>
-        <v>448.5</v>
+        <v>312</v>
       </c>
       <c r="D5" s="7" t="n">
         <f aca="false">Riepilogo!C5*(Parametri!$B$7+Parametri!$B$13)/Parametri!$B$7</f>
-        <v>12.4583333333333</v>
+        <v>13</v>
       </c>
       <c r="E5" s="28" t="n">
         <f aca="false">IF(Riepilogo!D5&gt;24,Parametri!$B$24,INDEX(Parametri!$B$21:$B$23,MATCH(D5,Parametri!$A$21:$A$23,1)))</f>
@@ -2929,264 +2501,210 @@
       </c>
       <c r="F5" s="7" t="n">
         <f aca="false">E5*Riepilogo!D5*Parametri!$B$12</f>
-        <v>1095.12</v>
+        <v>730.08</v>
       </c>
       <c r="G5" s="7" t="n">
         <f aca="false">Parametri!$B$15*Riepilogo!D5*Parametri!$B$12</f>
-        <v>28.08</v>
+        <v>18.72</v>
       </c>
       <c r="H5" s="7" t="n">
         <f aca="false">(B5+C5)/Parametri!$B$14</f>
-        <v>431.888888888889</v>
+        <v>300.444444444444</v>
       </c>
       <c r="I5" s="8" t="n">
         <f aca="false">B5+C5+F5+G5+H5</f>
-        <v>7385.58888888889</v>
+        <v>5105.24444444444</v>
       </c>
       <c r="J5" s="23" t="n">
         <f aca="false">Riepilogo!G5</f>
-        <v>5382</v>
+        <v>3744</v>
       </c>
       <c r="K5" s="8" t="n">
         <f aca="false">I5-J5</f>
-        <v>2003.58888888889</v>
+        <v>1361.24444444444</v>
       </c>
       <c r="L5" s="7" t="n">
         <f aca="false">K5/Parametri!$B$7</f>
-        <v>166.965740740741</v>
+        <v>113.437037037037</v>
       </c>
       <c r="M5" s="9" t="n">
         <f aca="false">IF(J5=0,0,K5/J5)</f>
-        <v>0.372275899087493</v>
+        <v>0.36358024691358</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="22" t="str">
         <f aca="false">Riepilogo!A6</f>
-        <v>Elisa</v>
+        <v>Corina</v>
       </c>
       <c r="B6" s="7" t="n">
         <f aca="false">Riepilogo!E6*Parametri!$B$12</f>
-        <v>3744</v>
+        <v>2080</v>
       </c>
       <c r="C6" s="7" t="n">
         <f aca="false">B6/Parametri!$B$7*Parametri!$B$13</f>
-        <v>312</v>
+        <v>173.333333333333</v>
       </c>
       <c r="D6" s="7" t="n">
         <f aca="false">Riepilogo!C6*(Parametri!$B$7+Parametri!$B$13)/Parametri!$B$7</f>
-        <v>13</v>
+        <v>10.8333333333333</v>
       </c>
       <c r="E6" s="28" t="n">
         <f aca="false">IF(Riepilogo!D6&gt;24,Parametri!$B$24,INDEX(Parametri!$B$21:$B$23,MATCH(D6,Parametri!$A$21:$A$23,1)))</f>
-        <v>2.34</v>
+        <v>1.92</v>
       </c>
       <c r="F6" s="7" t="n">
         <f aca="false">E6*Riepilogo!D6*Parametri!$B$12</f>
-        <v>730.08</v>
+        <v>399.36</v>
       </c>
       <c r="G6" s="7" t="n">
         <f aca="false">Parametri!$B$15*Riepilogo!D6*Parametri!$B$12</f>
-        <v>18.72</v>
+        <v>12.48</v>
       </c>
       <c r="H6" s="7" t="n">
         <f aca="false">(B6+C6)/Parametri!$B$14</f>
-        <v>300.444444444444</v>
+        <v>166.913580246914</v>
       </c>
       <c r="I6" s="8" t="n">
         <f aca="false">B6+C6+F6+G6+H6</f>
-        <v>5105.24444444444</v>
+        <v>2832.08691358025</v>
       </c>
       <c r="J6" s="23" t="n">
         <f aca="false">Riepilogo!G6</f>
-        <v>3744</v>
+        <v>2080</v>
       </c>
       <c r="K6" s="8" t="n">
         <f aca="false">I6-J6</f>
-        <v>1361.24444444444</v>
+        <v>752.086913580247</v>
       </c>
       <c r="L6" s="7" t="n">
         <f aca="false">K6/Parametri!$B$7</f>
-        <v>113.437037037037</v>
+        <v>62.6739094650206</v>
       </c>
       <c r="M6" s="9" t="n">
         <f aca="false">IF(J6=0,0,K6/J6)</f>
-        <v>0.36358024691358</v>
+        <v>0.36158024691358</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="22" t="str">
-        <f aca="false">Riepilogo!A7</f>
-        <v>Corina</v>
-      </c>
-      <c r="B7" s="7" t="n">
-        <f aca="false">Riepilogo!E7*Parametri!$B$12</f>
-        <v>2080</v>
-      </c>
-      <c r="C7" s="7" t="n">
-        <f aca="false">B7/Parametri!$B$7*Parametri!$B$13</f>
-        <v>173.333333333333</v>
-      </c>
-      <c r="D7" s="7" t="n">
-        <f aca="false">Riepilogo!C7*(Parametri!$B$7+Parametri!$B$13)/Parametri!$B$7</f>
-        <v>10.8333333333333</v>
-      </c>
-      <c r="E7" s="28" t="n">
-        <f aca="false">IF(Riepilogo!D7&gt;24,Parametri!$B$24,INDEX(Parametri!$B$21:$B$23,MATCH(D7,Parametri!$A$21:$A$23,1)))</f>
-        <v>1.92</v>
-      </c>
-      <c r="F7" s="7" t="n">
-        <f aca="false">E7*Riepilogo!D7*Parametri!$B$12</f>
-        <v>399.36</v>
-      </c>
-      <c r="G7" s="7" t="n">
-        <f aca="false">Parametri!$B$15*Riepilogo!D7*Parametri!$B$12</f>
-        <v>12.48</v>
-      </c>
-      <c r="H7" s="7" t="n">
-        <f aca="false">(B7+C7)/Parametri!$B$14</f>
-        <v>166.913580246914</v>
-      </c>
-      <c r="I7" s="8" t="n">
-        <f aca="false">B7+C7+F7+G7+H7</f>
-        <v>2832.08691358025</v>
-      </c>
-      <c r="J7" s="23" t="n">
-        <f aca="false">Riepilogo!G7</f>
-        <v>2080</v>
-      </c>
-      <c r="K7" s="8" t="n">
-        <f aca="false">I7-J7</f>
-        <v>752.086913580247</v>
-      </c>
-      <c r="L7" s="7" t="n">
-        <f aca="false">K7/Parametri!$B$7</f>
-        <v>62.6739094650206</v>
-      </c>
-      <c r="M7" s="9" t="n">
+      <c r="A7" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="11" t="n">
+        <f aca="false">SUM(B5:B6)</f>
+        <v>5824</v>
+      </c>
+      <c r="C7" s="11" t="n">
+        <f aca="false">SUM(C5:C6)</f>
+        <v>485.333333333333</v>
+      </c>
+      <c r="D7" s="10"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="11" t="n">
+        <f aca="false">SUM(F5:F6)</f>
+        <v>1129.44</v>
+      </c>
+      <c r="G7" s="11" t="n">
+        <f aca="false">SUM(G5:G6)</f>
+        <v>31.2</v>
+      </c>
+      <c r="H7" s="11" t="n">
+        <f aca="false">SUM(H5:H6)</f>
+        <v>467.358024691358</v>
+      </c>
+      <c r="I7" s="11" t="n">
+        <f aca="false">SUM(I5:I6)</f>
+        <v>7937.33135802469</v>
+      </c>
+      <c r="J7" s="11" t="n">
+        <f aca="false">SUM(J5:J6)</f>
+        <v>5824</v>
+      </c>
+      <c r="K7" s="11" t="n">
+        <f aca="false">SUM(K5:K6)</f>
+        <v>2113.33135802469</v>
+      </c>
+      <c r="L7" s="11" t="n">
+        <f aca="false">SUM(L5:L6)</f>
+        <v>176.110946502058</v>
+      </c>
+      <c r="M7" s="13" t="n">
         <f aca="false">IF(J7=0,0,K7/J7)</f>
-        <v>0.36158024691358</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="B8" s="11" t="n">
-        <f aca="false">SUM(B5:B7)</f>
-        <v>11206</v>
-      </c>
-      <c r="C8" s="11" t="n">
-        <f aca="false">SUM(C5:C7)</f>
-        <v>933.833333333333</v>
-      </c>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="11" t="n">
-        <f aca="false">SUM(F5:F7)</f>
-        <v>2224.56</v>
-      </c>
-      <c r="G8" s="11" t="n">
-        <f aca="false">SUM(G5:G7)</f>
-        <v>59.28</v>
-      </c>
-      <c r="H8" s="11" t="n">
-        <f aca="false">SUM(H5:H7)</f>
-        <v>899.246913580247</v>
-      </c>
-      <c r="I8" s="11" t="n">
-        <f aca="false">SUM(I5:I7)</f>
-        <v>15322.9202469136</v>
-      </c>
-      <c r="J8" s="11" t="n">
-        <f aca="false">SUM(J5:J7)</f>
-        <v>11206</v>
-      </c>
-      <c r="K8" s="11" t="n">
-        <f aca="false">SUM(K5:K7)</f>
-        <v>4116.92024691358</v>
-      </c>
-      <c r="L8" s="11" t="n">
-        <f aca="false">SUM(L5:L7)</f>
-        <v>343.076687242798</v>
-      </c>
-      <c r="M8" s="13" t="n">
-        <f aca="false">IF(J8=0,0,K8/J8)</f>
-        <v>0.367385351321933</v>
+        <v>0.362865961199295</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="14" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="14" t="s">
-        <v>97</v>
+      <c r="A11" s="15" t="s">
+        <v>96</v>
+      </c>
+      <c r="B11" s="8" t="n">
+        <f aca="false">(F7+G7)/4</f>
+        <v>290.16</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="15" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B12" s="8" t="n">
-        <f aca="false">(F8+G8)/4</f>
-        <v>570.96</v>
+        <f aca="false">H7/Parametri!$B$7</f>
+        <v>38.9465020576132</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="15" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B13" s="8" t="n">
-        <f aca="false">H8/Parametri!$B$7</f>
-        <v>74.9372427983539</v>
+        <f aca="false">C7</f>
+        <v>485.333333333333</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="B14" s="8" t="n">
+        <f aca="false">MIN(1549.37,(E5-INDEX(Parametri!$C$21:$C$23,MATCH(D5,Parametri!$A$21:$A$23,1)))*Riepilogo!D5*Parametri!$B$12+(E6-INDEX(Parametri!$C$21:$C$23,MATCH(D6,Parametri!$A$21:$A$23,1)))*Riepilogo!D6*Parametri!$B$12)</f>
+        <v>845.52</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="B14" s="8" t="n">
-        <f aca="false">C8</f>
-        <v>933.833333333333</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="15" t="s">
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="14" t="s">
         <v>101</v>
       </c>
-      <c r="B15" s="8" t="n">
-        <f aca="false">MIN(1549.37,(E5-INDEX(Parametri!$C$21:$C$23,MATCH(D5,Parametri!$A$21:$A$23,1)))*Riepilogo!D5*Parametri!$B$12+(E6-INDEX(Parametri!$C$21:$C$23,MATCH(D6,Parametri!$A$21:$A$23,1)))*Riepilogo!D6*Parametri!$B$12+(E7-INDEX(Parametri!$C$21:$C$23,MATCH(D7,Parametri!$A$21:$A$23,1)))*Riepilogo!D7*Parametri!$B$12)</f>
-        <v>1549.37</v>
-      </c>
-      <c r="C15" s="2" t="s">
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="17" t="s">
         <v>102</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="14" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="17" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="17" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="17" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="17" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="17" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
   </sheetData>

</xml_diff>